<commit_message>
test(bqs): reconcile v2 tank fixture and complete time log
</commit_message>
<xml_diff>
--- a/tests/fixtures/planilhas/bqs/synthetic-v2.xlsx
+++ b/tests/fixtures/planilhas/bqs/synthetic-v2.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="129">
   <si>
     <t>TEST company_contact</t>
   </si>
@@ -352,6 +352,12 @@
     <t>TEST sample_barge_surveyor</t>
   </si>
   <si>
+    <t>Operation</t>
+  </si>
+  <si>
+    <t>Test preparation</t>
+  </si>
+  <si>
     <t>Bunker Barge arrived</t>
   </si>
   <si>
@@ -395,6 +401,9 @@
   </si>
   <si>
     <t>Surveyor disembarked</t>
+  </si>
+  <si>
+    <t>Stoppages / Delays :</t>
   </si>
 </sst>
 </file>
@@ -1034,7 +1043,8 @@
         <v>10.125</v>
       </c>
       <c r="L20" s="1">
-        <v>11.125</v>
+        <f>0</f>
+        <v>0</v>
       </c>
       <c r="M20" s="1">
         <f>0</f>
@@ -1076,11 +1086,12 @@
         <v>10.125</v>
       </c>
       <c r="L21" s="1">
-        <v>11.125</v>
+        <f>112.25</f>
+        <v>112.25</v>
       </c>
       <c r="M21" s="1">
-        <f>0</f>
-        <v>0</v>
+        <f>111.125</f>
+        <v>111.125</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.25">
@@ -1118,7 +1129,8 @@
         <v>10.125</v>
       </c>
       <c r="L22" s="1">
-        <v>11.125</v>
+        <f>0</f>
+        <v>0</v>
       </c>
       <c r="M22" s="1">
         <f>0</f>
@@ -1160,7 +1172,8 @@
         <v>10.125</v>
       </c>
       <c r="L23" s="1">
-        <v>11.125</v>
+        <f>0</f>
+        <v>0</v>
       </c>
       <c r="M23" s="1">
         <f>0</f>
@@ -1202,7 +1215,8 @@
         <v>10.125</v>
       </c>
       <c r="L24" s="1">
-        <v>11.125</v>
+        <f>0</f>
+        <v>0</v>
       </c>
       <c r="M24" s="1">
         <f>0</f>
@@ -1244,7 +1258,8 @@
         <v>10.125</v>
       </c>
       <c r="L25" s="1">
-        <v>11.125</v>
+        <f>0</f>
+        <v>0</v>
       </c>
       <c r="M25" s="1">
         <f>0</f>
@@ -1286,7 +1301,8 @@
         <v>10.125</v>
       </c>
       <c r="L26" s="1">
-        <v>11.125</v>
+        <f>0</f>
+        <v>0</v>
       </c>
       <c r="M26" s="1">
         <f>0</f>
@@ -1328,7 +1344,8 @@
         <v>10.125</v>
       </c>
       <c r="L27" s="1">
-        <v>11.125</v>
+        <f>0</f>
+        <v>0</v>
       </c>
       <c r="M27" s="1">
         <f>0</f>
@@ -1370,7 +1387,8 @@
         <v>10.125</v>
       </c>
       <c r="L28" s="1">
-        <v>11.125</v>
+        <f>0</f>
+        <v>0</v>
       </c>
       <c r="M28" s="1">
         <f>0</f>
@@ -1412,7 +1430,8 @@
         <v>10.125</v>
       </c>
       <c r="L29" s="1">
-        <v>11.125</v>
+        <f>0</f>
+        <v>0</v>
       </c>
       <c r="M29" s="1">
         <f>0</f>
@@ -1454,7 +1473,8 @@
         <v>10.125</v>
       </c>
       <c r="L30" s="1">
-        <v>11.125</v>
+        <f>0</f>
+        <v>0</v>
       </c>
       <c r="M30" s="1">
         <f>0</f>
@@ -1496,7 +1516,8 @@
         <v>10.125</v>
       </c>
       <c r="L31" s="1">
-        <v>11.125</v>
+        <f>0</f>
+        <v>0</v>
       </c>
       <c r="M31" s="1">
         <f>0</f>
@@ -1538,7 +1559,8 @@
         <v>10.125</v>
       </c>
       <c r="L32" s="1">
-        <v>11.125</v>
+        <f>0</f>
+        <v>0</v>
       </c>
       <c r="M32" s="1">
         <f>0</f>
@@ -1580,7 +1602,8 @@
         <v>10.125</v>
       </c>
       <c r="L33" s="1">
-        <v>11.125</v>
+        <f>0</f>
+        <v>0</v>
       </c>
       <c r="M33" s="1">
         <f>0</f>
@@ -1622,7 +1645,8 @@
         <v>10.125</v>
       </c>
       <c r="L34" s="1">
-        <v>11.125</v>
+        <f>0</f>
+        <v>0</v>
       </c>
       <c r="M34" s="1">
         <f>0</f>
@@ -1664,7 +1688,8 @@
         <v>10.125</v>
       </c>
       <c r="L35" s="1">
-        <v>11.125</v>
+        <f>0</f>
+        <v>0</v>
       </c>
       <c r="M35" s="1">
         <f>0</f>
@@ -1706,7 +1731,8 @@
         <v>10.125</v>
       </c>
       <c r="L36" s="1">
-        <v>11.125</v>
+        <f>0</f>
+        <v>0</v>
       </c>
       <c r="M36" s="1">
         <f>0</f>
@@ -1748,7 +1774,8 @@
         <v>10.125</v>
       </c>
       <c r="L37" s="1">
-        <v>11.125</v>
+        <f>0</f>
+        <v>0</v>
       </c>
       <c r="M37" s="1">
         <f>0</f>
@@ -1790,7 +1817,8 @@
         <v>10.125</v>
       </c>
       <c r="L38" s="1">
-        <v>11.125</v>
+        <f>0</f>
+        <v>0</v>
       </c>
       <c r="M38" s="1">
         <f>0</f>
@@ -1832,7 +1860,8 @@
         <v>10.125</v>
       </c>
       <c r="L39" s="1">
-        <v>11.125</v>
+        <f>0</f>
+        <v>0</v>
       </c>
       <c r="M39" s="1">
         <f>0</f>
@@ -1874,7 +1903,8 @@
         <v>10.125</v>
       </c>
       <c r="L40" s="1">
-        <v>11.125</v>
+        <f>0</f>
+        <v>0</v>
       </c>
       <c r="M40" s="1">
         <f>0</f>
@@ -1916,7 +1946,8 @@
         <v>10.125</v>
       </c>
       <c r="L41" s="1">
-        <v>11.125</v>
+        <f>0</f>
+        <v>0</v>
       </c>
       <c r="M41" s="1">
         <f>0</f>
@@ -1958,7 +1989,8 @@
         <v>10.125</v>
       </c>
       <c r="L42" s="1">
-        <v>11.125</v>
+        <f>0</f>
+        <v>0</v>
       </c>
       <c r="M42" s="1">
         <f>0</f>
@@ -2000,7 +2032,8 @@
         <v>10.125</v>
       </c>
       <c r="L43" s="1">
-        <v>11.125</v>
+        <f>0</f>
+        <v>0</v>
       </c>
       <c r="M43" s="1">
         <f>0</f>
@@ -2042,7 +2075,8 @@
         <v>10.125</v>
       </c>
       <c r="L44" s="1">
-        <v>11.125</v>
+        <f>0</f>
+        <v>0</v>
       </c>
       <c r="M44" s="1">
         <f>0</f>
@@ -2108,7 +2142,8 @@
         <v>10.125</v>
       </c>
       <c r="L53" s="1">
-        <v>11.125</v>
+        <f>0</f>
+        <v>0</v>
       </c>
       <c r="M53" s="1">
         <f>0</f>
@@ -2150,11 +2185,12 @@
         <v>10.125</v>
       </c>
       <c r="L54" s="1">
-        <v>11.125</v>
+        <f>446.5</f>
+        <v>446.5</v>
       </c>
       <c r="M54" s="1">
-        <f>0</f>
-        <v>0</v>
+        <f>444.875</f>
+        <v>444.875</v>
       </c>
     </row>
     <row r="55" spans="1:13" x14ac:dyDescent="0.25">
@@ -2192,7 +2228,8 @@
         <v>10.125</v>
       </c>
       <c r="L55" s="1">
-        <v>11.125</v>
+        <f>0</f>
+        <v>0</v>
       </c>
       <c r="M55" s="1">
         <f>0</f>
@@ -2234,7 +2271,8 @@
         <v>10.125</v>
       </c>
       <c r="L56" s="1">
-        <v>11.125</v>
+        <f>0</f>
+        <v>0</v>
       </c>
       <c r="M56" s="1">
         <f>0</f>
@@ -2276,7 +2314,8 @@
         <v>10.125</v>
       </c>
       <c r="L57" s="1">
-        <v>11.125</v>
+        <f>0</f>
+        <v>0</v>
       </c>
       <c r="M57" s="1">
         <f>0</f>
@@ -2318,7 +2357,8 @@
         <v>10.125</v>
       </c>
       <c r="L58" s="1">
-        <v>11.125</v>
+        <f>0</f>
+        <v>0</v>
       </c>
       <c r="M58" s="1">
         <f>0</f>
@@ -2360,7 +2400,8 @@
         <v>10.125</v>
       </c>
       <c r="L59" s="1">
-        <v>11.125</v>
+        <f>0</f>
+        <v>0</v>
       </c>
       <c r="M59" s="1">
         <f>0</f>
@@ -2402,7 +2443,8 @@
         <v>10.125</v>
       </c>
       <c r="L60" s="1">
-        <v>11.125</v>
+        <f>0</f>
+        <v>0</v>
       </c>
       <c r="M60" s="1">
         <f>0</f>
@@ -2444,7 +2486,8 @@
         <v>10.125</v>
       </c>
       <c r="L61" s="1">
-        <v>11.125</v>
+        <f>0</f>
+        <v>0</v>
       </c>
       <c r="M61" s="1">
         <f>0</f>
@@ -2486,7 +2529,8 @@
         <v>10.125</v>
       </c>
       <c r="L62" s="1">
-        <v>11.125</v>
+        <f>0</f>
+        <v>0</v>
       </c>
       <c r="M62" s="1">
         <f>0</f>
@@ -2528,7 +2572,8 @@
         <v>10.125</v>
       </c>
       <c r="L63" s="1">
-        <v>11.125</v>
+        <f>0</f>
+        <v>0</v>
       </c>
       <c r="M63" s="1">
         <f>0</f>
@@ -2570,7 +2615,8 @@
         <v>10.125</v>
       </c>
       <c r="L64" s="1">
-        <v>11.125</v>
+        <f>0</f>
+        <v>0</v>
       </c>
       <c r="M64" s="1">
         <f>0</f>
@@ -2612,7 +2658,8 @@
         <v>10.125</v>
       </c>
       <c r="L65" s="1">
-        <v>11.125</v>
+        <f>0</f>
+        <v>0</v>
       </c>
       <c r="M65" s="1">
         <f>0</f>
@@ -2654,7 +2701,8 @@
         <v>10.125</v>
       </c>
       <c r="L66" s="1">
-        <v>11.125</v>
+        <f>0</f>
+        <v>0</v>
       </c>
       <c r="M66" s="1">
         <f>0</f>
@@ -2696,7 +2744,8 @@
         <v>10.125</v>
       </c>
       <c r="L67" s="1">
-        <v>11.125</v>
+        <f>0</f>
+        <v>0</v>
       </c>
       <c r="M67" s="1">
         <f>0</f>
@@ -2738,7 +2787,8 @@
         <v>10.125</v>
       </c>
       <c r="L68" s="1">
-        <v>11.125</v>
+        <f>0</f>
+        <v>0</v>
       </c>
       <c r="M68" s="1">
         <f>0</f>
@@ -2780,7 +2830,8 @@
         <v>10.125</v>
       </c>
       <c r="L69" s="1">
-        <v>11.125</v>
+        <f>0</f>
+        <v>0</v>
       </c>
       <c r="M69" s="1">
         <f>0</f>
@@ -2822,7 +2873,8 @@
         <v>10.125</v>
       </c>
       <c r="L70" s="1">
-        <v>11.125</v>
+        <f>0</f>
+        <v>0</v>
       </c>
       <c r="M70" s="1">
         <f>0</f>
@@ -2864,7 +2916,8 @@
         <v>10.125</v>
       </c>
       <c r="L71" s="1">
-        <v>11.125</v>
+        <f>0</f>
+        <v>0</v>
       </c>
       <c r="M71" s="1">
         <f>0</f>
@@ -2989,7 +3042,8 @@
         <v>10.125</v>
       </c>
       <c r="M20" s="1">
-        <v>11.125</v>
+        <f>0</f>
+        <v>0</v>
       </c>
       <c r="N20" s="1">
         <f>0</f>
@@ -3031,11 +3085,12 @@
         <v>10.125</v>
       </c>
       <c r="M21" s="1">
-        <v>11.125</v>
+        <f>902.5</f>
+        <v>902.5</v>
       </c>
       <c r="N21" s="1">
-        <f>0</f>
-        <v>0</v>
+        <f>900.75</f>
+        <v>900.75</v>
       </c>
     </row>
     <row r="22" spans="2:14" x14ac:dyDescent="0.25">
@@ -3073,7 +3128,8 @@
         <v>10.125</v>
       </c>
       <c r="M22" s="1">
-        <v>11.125</v>
+        <f>0</f>
+        <v>0</v>
       </c>
       <c r="N22" s="1">
         <f>0</f>
@@ -3115,7 +3171,8 @@
         <v>10.125</v>
       </c>
       <c r="M23" s="1">
-        <v>11.125</v>
+        <f>0</f>
+        <v>0</v>
       </c>
       <c r="N23" s="1">
         <f>0</f>
@@ -3157,7 +3214,8 @@
         <v>10.125</v>
       </c>
       <c r="M24" s="1">
-        <v>11.125</v>
+        <f>0</f>
+        <v>0</v>
       </c>
       <c r="N24" s="1">
         <f>0</f>
@@ -3199,7 +3257,8 @@
         <v>10.125</v>
       </c>
       <c r="M25" s="1">
-        <v>11.125</v>
+        <f>0</f>
+        <v>0</v>
       </c>
       <c r="N25" s="1">
         <f>0</f>
@@ -3241,7 +3300,8 @@
         <v>10.125</v>
       </c>
       <c r="M26" s="1">
-        <v>11.125</v>
+        <f>0</f>
+        <v>0</v>
       </c>
       <c r="N26" s="1">
         <f>0</f>
@@ -3283,7 +3343,8 @@
         <v>10.125</v>
       </c>
       <c r="M27" s="1">
-        <v>11.125</v>
+        <f>0</f>
+        <v>0</v>
       </c>
       <c r="N27" s="1">
         <f>0</f>
@@ -3354,7 +3415,8 @@
         <v>10.125</v>
       </c>
       <c r="M35" s="1">
-        <v>11.125</v>
+        <f>0</f>
+        <v>0</v>
       </c>
       <c r="N35" s="1">
         <f>0</f>
@@ -3396,11 +3458,12 @@
         <v>10.125</v>
       </c>
       <c r="M36" s="1">
-        <v>11.125</v>
+        <f>580</f>
+        <v>580</v>
       </c>
       <c r="N36" s="1">
-        <f>0</f>
-        <v>0</v>
+        <f>578.25</f>
+        <v>578.25</v>
       </c>
     </row>
     <row r="37" spans="2:14" x14ac:dyDescent="0.25">
@@ -3438,7 +3501,8 @@
         <v>10.125</v>
       </c>
       <c r="M37" s="1">
-        <v>11.125</v>
+        <f>0</f>
+        <v>0</v>
       </c>
       <c r="N37" s="1">
         <f>0</f>
@@ -3480,7 +3544,8 @@
         <v>10.125</v>
       </c>
       <c r="M38" s="1">
-        <v>11.125</v>
+        <f>0</f>
+        <v>0</v>
       </c>
       <c r="N38" s="1">
         <f>0</f>
@@ -3522,7 +3587,8 @@
         <v>10.125</v>
       </c>
       <c r="M39" s="1">
-        <v>11.125</v>
+        <f>0</f>
+        <v>0</v>
       </c>
       <c r="N39" s="1">
         <f>0</f>
@@ -3564,7 +3630,8 @@
         <v>10.125</v>
       </c>
       <c r="M40" s="1">
-        <v>11.125</v>
+        <f>0</f>
+        <v>0</v>
       </c>
       <c r="N40" s="1">
         <f>0</f>
@@ -3606,7 +3673,8 @@
         <v>10.125</v>
       </c>
       <c r="M41" s="1">
-        <v>11.125</v>
+        <f>0</f>
+        <v>0</v>
       </c>
       <c r="N41" s="1">
         <f>0</f>
@@ -3648,7 +3716,8 @@
         <v>10.125</v>
       </c>
       <c r="M42" s="1">
-        <v>11.125</v>
+        <f>0</f>
+        <v>0</v>
       </c>
       <c r="N42" s="1">
         <f>0</f>
@@ -3797,133 +3866,154 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A19:F32"/>
+  <dimension ref="A15:F35"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>112</v>
+      </c>
+      <c r="D16" t="s">
+        <v>11</v>
+      </c>
+      <c r="E16">
+        <v>0</v>
+      </c>
+    </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="D19" t="s">
         <v>11</v>
       </c>
       <c r="E19" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="F19" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D20" t="s">
         <v>11</v>
       </c>
       <c r="E20" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="F20" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D21" t="s">
         <v>11</v>
       </c>
       <c r="E21" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="F21" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="D22" t="s">
         <v>11</v>
       </c>
       <c r="E22" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="F22" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="D24" t="s">
         <v>11</v>
       </c>
       <c r="E24" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="F24" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="D26" t="s">
         <v>11</v>
       </c>
       <c r="E26" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="F26" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="D27" t="s">
         <v>11</v>
       </c>
       <c r="E27" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="F27" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="D28" t="s">
         <v>11</v>
       </c>
       <c r="E28" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="F28" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="D32" t="s">
         <v>11</v>
       </c>
       <c r="E32" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="F32" t="s">
-        <v>112</v>
+        <v>114</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>128</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(bqs): preserve LOA text and typecheck v2 fixtures
</commit_message>
<xml_diff>
--- a/tests/fixtures/planilhas/bqs/synthetic-v2.xlsx
+++ b/tests/fixtures/planilhas/bqs/synthetic-v2.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="142">
   <si>
     <t>TEST company_contact</t>
   </si>
@@ -52,6 +52,9 @@
     <t>TEST vessel_delivered</t>
   </si>
   <si>
+    <t>229.00</t>
+  </si>
+  <si>
     <t>10/05/2026</t>
   </si>
   <si>
@@ -361,15 +364,30 @@
     <t>Bunker Barge arrived</t>
   </si>
   <si>
+    <t>16:20</t>
+  </si>
+  <si>
+    <t>16:25</t>
+  </si>
+  <si>
+    <t>Surveyor embarked</t>
+  </si>
+  <si>
+    <t>16:30</t>
+  </si>
+  <si>
+    <t>16:35</t>
+  </si>
+  <si>
+    <t>Meeting between Chief Engineer and Surveyor</t>
+  </si>
+  <si>
+    <t>16:40</t>
+  </si>
+  <si>
     <t>17:00</t>
   </si>
   <si>
-    <t>Surveyor embarked</t>
-  </si>
-  <si>
-    <t>Meeting between Chief Engineer and Surveyor</t>
-  </si>
-  <si>
     <t>Initial soundings / Ullage - Vessel</t>
   </si>
   <si>
@@ -385,22 +403,43 @@
     <t>18:03</t>
   </si>
   <si>
+    <t>18:27</t>
+  </si>
+  <si>
     <t>Bunkering operation</t>
   </si>
   <si>
+    <t>18:45</t>
+  </si>
+  <si>
+    <t>21:50</t>
+  </si>
+  <si>
     <t>Final soundings / Ullage - Barge</t>
   </si>
   <si>
     <t>22:04</t>
   </si>
   <si>
+    <t>22:19</t>
+  </si>
+  <si>
     <t>Final soundings / Ullage - Vessel</t>
   </si>
   <si>
     <t>22:23</t>
   </si>
   <si>
+    <t>22:47</t>
+  </si>
+  <si>
     <t>Surveyor disembarked</t>
+  </si>
+  <si>
+    <t>23:10</t>
+  </si>
+  <si>
+    <t>23:15</t>
   </si>
   <si>
     <t>Stoppages / Delays :</t>
@@ -843,28 +882,28 @@
       </c>
     </row>
     <row r="21" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C21">
-        <v>0</v>
+      <c r="C21" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="23" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C23" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="25" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C25" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="26" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C26" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="27" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C27" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="28" spans="3:5" x14ac:dyDescent="0.25">
@@ -879,52 +918,52 @@
     </row>
     <row r="30" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C30" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="31" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C31" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="33" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C33" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="34" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C34" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="36" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C36" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="37" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C37" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="40" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C40" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="41" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C41" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="42" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C42" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="43" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C43" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="44" spans="3:3" x14ac:dyDescent="0.25">
@@ -939,17 +978,17 @@
     </row>
     <row r="46" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C46" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="48" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C48" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="49" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C49" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
   </sheetData>
@@ -965,33 +1004,33 @@
   <sheetData>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="8" spans="3:9" x14ac:dyDescent="0.25">
       <c r="C8" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="I8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="9" spans="9:9" x14ac:dyDescent="0.25">
       <c r="I9" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="10" spans="3:9" x14ac:dyDescent="0.25">
       <c r="C10" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="I10" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="11" spans="9:9" x14ac:dyDescent="0.25">
       <c r="I11" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="17" spans="2:11" x14ac:dyDescent="0.25">
@@ -1005,15 +1044,15 @@
         <v>0</v>
       </c>
       <c r="K17" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C20" s="1">
         <v>2.125</v>
@@ -1053,10 +1092,10 @@
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C21" s="1">
         <v>2.125</v>
@@ -1096,10 +1135,10 @@
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C22" s="1">
         <v>2.125</v>
@@ -1139,10 +1178,10 @@
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C23" s="1">
         <v>2.125</v>
@@ -1182,10 +1221,10 @@
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C24" s="1">
         <v>2.125</v>
@@ -1225,10 +1264,10 @@
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C25" s="1">
         <v>2.125</v>
@@ -1268,10 +1307,10 @@
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C26" s="1">
         <v>2.125</v>
@@ -1311,10 +1350,10 @@
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C27" s="1">
         <v>2.125</v>
@@ -1354,10 +1393,10 @@
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C28" s="1">
         <v>2.125</v>
@@ -1397,10 +1436,10 @@
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C29" s="1">
         <v>2.125</v>
@@ -1440,10 +1479,10 @@
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C30" s="1">
         <v>2.125</v>
@@ -1483,10 +1522,10 @@
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C31" s="1">
         <v>2.125</v>
@@ -1526,10 +1565,10 @@
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C32" s="1">
         <v>2.125</v>
@@ -1569,10 +1608,10 @@
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C33" s="1">
         <v>2.125</v>
@@ -1612,10 +1651,10 @@
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C34" s="1">
         <v>2.125</v>
@@ -1655,10 +1694,10 @@
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C35" s="1">
         <v>2.125</v>
@@ -1698,10 +1737,10 @@
     </row>
     <row r="36" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C36" s="1">
         <v>2.125</v>
@@ -1741,10 +1780,10 @@
     </row>
     <row r="37" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C37" s="1">
         <v>2.125</v>
@@ -1784,10 +1823,10 @@
     </row>
     <row r="38" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C38" s="1">
         <v>2.125</v>
@@ -1827,10 +1866,10 @@
     </row>
     <row r="39" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C39" s="1">
         <v>2.125</v>
@@ -1870,10 +1909,10 @@
     </row>
     <row r="40" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C40" s="1">
         <v>2.125</v>
@@ -1913,10 +1952,10 @@
     </row>
     <row r="41" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C41" s="1">
         <v>2.125</v>
@@ -1956,10 +1995,10 @@
     </row>
     <row r="42" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C42" s="1">
         <v>2.125</v>
@@ -1999,10 +2038,10 @@
     </row>
     <row r="43" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C43" s="1">
         <v>2.125</v>
@@ -2042,10 +2081,10 @@
     </row>
     <row r="44" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C44" s="1">
         <v>2.125</v>
@@ -2104,15 +2143,15 @@
         <v>0</v>
       </c>
       <c r="K50" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="53" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C53" s="1">
         <v>2.125</v>
@@ -2152,10 +2191,10 @@
     </row>
     <row r="54" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C54" s="1">
         <v>2.125</v>
@@ -2195,10 +2234,10 @@
     </row>
     <row r="55" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C55" s="1">
         <v>2.125</v>
@@ -2238,10 +2277,10 @@
     </row>
     <row r="56" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C56" s="1">
         <v>2.125</v>
@@ -2281,10 +2320,10 @@
     </row>
     <row r="57" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C57" s="1">
         <v>2.125</v>
@@ -2324,10 +2363,10 @@
     </row>
     <row r="58" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C58" s="1">
         <v>2.125</v>
@@ -2367,10 +2406,10 @@
     </row>
     <row r="59" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C59" s="1">
         <v>2.125</v>
@@ -2410,10 +2449,10 @@
     </row>
     <row r="60" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C60" s="1">
         <v>2.125</v>
@@ -2453,10 +2492,10 @@
     </row>
     <row r="61" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C61" s="1">
         <v>2.125</v>
@@ -2496,10 +2535,10 @@
     </row>
     <row r="62" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C62" s="1">
         <v>2.125</v>
@@ -2539,10 +2578,10 @@
     </row>
     <row r="63" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C63" s="1">
         <v>2.125</v>
@@ -2582,10 +2621,10 @@
     </row>
     <row r="64" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C64" s="1">
         <v>2.125</v>
@@ -2625,10 +2664,10 @@
     </row>
     <row r="65" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C65" s="1">
         <v>2.125</v>
@@ -2668,10 +2707,10 @@
     </row>
     <row r="66" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A66" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C66" s="1">
         <v>2.125</v>
@@ -2711,10 +2750,10 @@
     </row>
     <row r="67" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C67" s="1">
         <v>2.125</v>
@@ -2754,10 +2793,10 @@
     </row>
     <row r="68" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A68" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C68" s="1">
         <v>2.125</v>
@@ -2797,10 +2836,10 @@
     </row>
     <row r="69" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A69" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C69" s="1">
         <v>2.125</v>
@@ -2840,10 +2879,10 @@
     </row>
     <row r="70" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A70" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C70" s="1">
         <v>2.125</v>
@@ -2883,10 +2922,10 @@
     </row>
     <row r="71" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A71" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C71" s="1">
         <v>2.125</v>
@@ -2936,12 +2975,12 @@
     </row>
     <row r="76" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C76" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="77" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C77" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="L77">
         <f>335.25</f>
@@ -2956,7 +2995,7 @@
     </row>
     <row r="79" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C79" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="L79">
         <f>-1.5</f>
@@ -2971,10 +3010,10 @@
     </row>
     <row r="93" spans="4:11" x14ac:dyDescent="0.25">
       <c r="D93" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="K93" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
   </sheetData>
@@ -2990,7 +3029,7 @@
   <sheetData>
     <row r="16" spans="11:11" x14ac:dyDescent="0.25">
       <c r="K16" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="17" spans="3:12" x14ac:dyDescent="0.25">
@@ -3004,15 +3043,15 @@
         <v>0</v>
       </c>
       <c r="L17" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="20" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B20" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D20" s="1">
         <v>2.125</v>
@@ -3052,10 +3091,10 @@
     </row>
     <row r="21" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B21" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D21" s="1">
         <v>2.125</v>
@@ -3095,10 +3134,10 @@
     </row>
     <row r="22" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B22" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D22" s="1">
         <v>2.125</v>
@@ -3138,10 +3177,10 @@
     </row>
     <row r="23" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B23" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D23" s="1">
         <v>2.125</v>
@@ -3181,10 +3220,10 @@
     </row>
     <row r="24" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B24" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D24" s="1">
         <v>2.125</v>
@@ -3224,10 +3263,10 @@
     </row>
     <row r="25" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B25" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D25" s="1">
         <v>2.125</v>
@@ -3267,10 +3306,10 @@
     </row>
     <row r="26" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B26" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D26" s="1">
         <v>2.125</v>
@@ -3310,10 +3349,10 @@
     </row>
     <row r="27" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B27" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D27" s="1">
         <v>2.125</v>
@@ -3363,7 +3402,7 @@
     </row>
     <row r="31" spans="11:11" x14ac:dyDescent="0.25">
       <c r="K31" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="32" spans="3:12" x14ac:dyDescent="0.25">
@@ -3377,15 +3416,15 @@
         <v>0</v>
       </c>
       <c r="L32" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="35" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B35" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D35" s="1">
         <v>2.125</v>
@@ -3425,10 +3464,10 @@
     </row>
     <row r="36" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B36" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D36" s="1">
         <v>2.125</v>
@@ -3468,10 +3507,10 @@
     </row>
     <row r="37" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B37" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D37" s="1">
         <v>2.125</v>
@@ -3511,10 +3550,10 @@
     </row>
     <row r="38" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B38" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D38" s="1">
         <v>2.125</v>
@@ -3554,10 +3593,10 @@
     </row>
     <row r="39" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B39" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D39" s="1">
         <v>2.125</v>
@@ -3597,10 +3636,10 @@
     </row>
     <row r="40" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B40" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D40" s="1">
         <v>2.125</v>
@@ -3640,10 +3679,10 @@
     </row>
     <row r="41" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B41" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D41" s="1">
         <v>2.125</v>
@@ -3683,10 +3722,10 @@
     </row>
     <row r="42" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B42" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D42" s="1">
         <v>2.125</v>
@@ -3760,25 +3799,25 @@
     </row>
     <row r="50" spans="4:13" x14ac:dyDescent="0.25">
       <c r="D50" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="M50" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="51" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D51" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="52" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D52" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="54" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D54" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
   </sheetData>
@@ -3794,68 +3833,68 @@
   <sheetData>
     <row r="21" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D21" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="22" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D22" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="23" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D23" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="F23" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="24" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D24" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="F24" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="26" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D26" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="F26" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="27" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D27" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="F27" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="28" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D28" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="F28" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="29" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D29" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F29" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="30" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D30" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F30" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
   </sheetData>
@@ -3871,15 +3910,15 @@
   <sheetData>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D16" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E16">
         <v>0</v>
@@ -3887,133 +3926,133 @@
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D19" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E19" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="F19" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="D20" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E20" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="F20" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="D21" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E21" t="s">
-        <v>114</v>
+        <v>121</v>
       </c>
       <c r="F21" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="D22" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E22" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="F22" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="D24" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E24" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="F24" t="s">
-        <v>114</v>
+        <v>128</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>122</v>
+        <v>129</v>
       </c>
       <c r="D26" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E26" t="s">
-        <v>114</v>
+        <v>130</v>
       </c>
       <c r="F26" t="s">
-        <v>114</v>
+        <v>131</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>123</v>
+        <v>132</v>
       </c>
       <c r="D27" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E27" t="s">
-        <v>124</v>
+        <v>133</v>
       </c>
       <c r="F27" t="s">
-        <v>114</v>
+        <v>134</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>125</v>
+        <v>135</v>
       </c>
       <c r="D28" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E28" t="s">
-        <v>126</v>
+        <v>136</v>
       </c>
       <c r="F28" t="s">
-        <v>114</v>
+        <v>137</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>127</v>
+        <v>138</v>
       </c>
       <c r="D32" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E32" t="s">
-        <v>114</v>
+        <v>139</v>
       </c>
       <c r="F32" t="s">
-        <v>114</v>
+        <v>140</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>128</v>
+        <v>141</v>
       </c>
     </row>
   </sheetData>

</xml_diff>